<commit_message>
Changed the explorer algorithm to match exact instances in the statguide table column 0. Stemming is discarded. Now a secondary algorithm remains that finds all alternative representations that are associated with each individual terms. Based on 'pivot words' (in Cox Regression analysis this will be cox) the algorithm should return bi, tri and tetragrams with this pivot word included; thereby generating the required alternative representations that are both specific and sensitive to the respective concept.
</commit_message>
<xml_diff>
--- a/input/StatGuide.xlsx
+++ b/input/StatGuide.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yannic/Dropbox/Code/Static V2/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yannic/Dropbox/Code/StatAssist_V2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2076AEB-5B44-604F-AEE6-97895A0B2C35}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5E60F48-AB6A-494C-A0BD-3E3E9A026513}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12560" yWindow="8220" windowWidth="23540" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -966,9 +966,6 @@
 In the end, it is up to the analyst to determine what the meaning of an outlier is; high variability or just experimental error.</t>
   </si>
   <si>
-    <t>P-value</t>
-  </si>
-  <si>
     <t>P-Value</t>
   </si>
   <si>
@@ -1578,6 +1575,9 @@
   </si>
   <si>
     <t>What does it mean?</t>
+  </si>
+  <si>
+    <t>p</t>
   </si>
 </sst>
 </file>
@@ -2053,19 +2053,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
@@ -2219,7 +2219,7 @@
       <c r="X6" s="4"/>
       <c r="Y6" s="4"/>
     </row>
-    <row r="7" spans="1:25" ht="306">
+    <row r="7" spans="1:25" ht="409.6">
       <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>173</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F42" s="7"/>
       <c r="G42" s="7" t="s">
@@ -3452,7 +3452,7 @@
         <v>190</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="7" t="s">
@@ -3558,7 +3558,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="398">
+    <row r="52" spans="1:7" ht="409.6">
       <c r="A52" s="7" t="s">
         <v>219</v>
       </c>
@@ -3900,30 +3900,30 @@
     </row>
     <row r="70" spans="1:7" ht="210">
       <c r="A70" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="B70" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="B70" s="7" t="s">
+      <c r="C70" s="7" t="s">
         <v>303</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>304</v>
       </c>
       <c r="D70" s="7"/>
       <c r="E70" s="8"/>
       <c r="F70" s="7"/>
       <c r="G70" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="60">
       <c r="A71" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="C71" s="7" t="s">
         <v>306</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>307</v>
       </c>
       <c r="D71" s="7"/>
       <c r="E71" s="8"/>
@@ -3932,97 +3932,97 @@
     </row>
     <row r="72" spans="1:7" ht="285">
       <c r="A72" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="C72" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="C72" s="10" t="s">
+      <c r="D72" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="D72" s="7" t="s">
-        <v>311</v>
-      </c>
       <c r="E72" s="8" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="120">
       <c r="A73" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="C73" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="B73" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="C73" s="7" t="s">
+      <c r="D73" s="7" t="s">
         <v>314</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>315</v>
       </c>
       <c r="E73" s="8"/>
       <c r="F73" s="7"/>
       <c r="G73" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="105">
       <c r="A74" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="B74" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="B74" s="7" t="s">
+      <c r="C74" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="C74" s="10" t="s">
+      <c r="D74" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="D74" s="7" t="s">
-        <v>320</v>
-      </c>
       <c r="E74" s="8" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F74" s="7"/>
       <c r="G74" s="7" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="409.6">
+      <c r="A75" s="7" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" ht="398">
-      <c r="A75" s="7" t="s">
+      <c r="B75" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="C75" s="7" t="s">
         <v>323</v>
       </c>
-      <c r="C75" s="7" t="s">
+      <c r="D75" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="D75" s="7" t="s">
+      <c r="E75" s="8" t="s">
+        <v>483</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="G75" s="7" t="s">
         <v>325</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>484</v>
-      </c>
-      <c r="F75" s="7" t="s">
-        <v>327</v>
-      </c>
-      <c r="G75" s="7" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="75">
       <c r="A76" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C76" s="7" t="s">
         <v>328</v>
-      </c>
-      <c r="B76" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="C76" s="7" t="s">
-        <v>329</v>
       </c>
       <c r="D76" s="7"/>
       <c r="E76" s="8"/>
@@ -4031,92 +4031,92 @@
     </row>
     <row r="77" spans="1:7" ht="90">
       <c r="A77" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="B77" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="B77" s="7" t="s">
+      <c r="C77" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="D77" s="7" t="s">
         <v>332</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>333</v>
       </c>
       <c r="E77" s="8"/>
       <c r="F77" s="7"/>
       <c r="G77" s="7" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="120">
       <c r="A78" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="C78" s="7" t="s">
         <v>335</v>
       </c>
-      <c r="B78" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="C78" s="7" t="s">
+      <c r="D78" s="7" t="s">
         <v>336</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>337</v>
       </c>
       <c r="E78" s="8"/>
       <c r="F78" s="7"/>
       <c r="G78" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="75">
       <c r="A79" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="C79" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="B79" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="C79" s="7" t="s">
+      <c r="D79" s="7" t="s">
         <v>340</v>
-      </c>
-      <c r="D79" s="7" t="s">
-        <v>341</v>
       </c>
       <c r="E79" s="8"/>
       <c r="F79" s="7"/>
       <c r="G79" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="384">
       <c r="A80" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B80" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="C80" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="D80" s="7" t="s">
         <v>345</v>
-      </c>
-      <c r="D80" s="7" t="s">
-        <v>346</v>
       </c>
       <c r="E80" s="8"/>
       <c r="F80" s="7"/>
       <c r="G80" s="7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="342">
       <c r="A81" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B81" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="B81" s="7" t="s">
+      <c r="C81" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="C81" s="7" t="s">
+      <c r="D81" s="7" t="s">
         <v>350</v>
-      </c>
-      <c r="D81" s="7" t="s">
-        <v>351</v>
       </c>
       <c r="E81" s="8"/>
       <c r="F81" s="7"/>
@@ -4124,121 +4124,121 @@
     </row>
     <row r="82" spans="1:7" ht="84">
       <c r="A82" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="C82" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="B82" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="C82" s="7" t="s">
+      <c r="D82" s="11" t="s">
         <v>353</v>
-      </c>
-      <c r="D82" s="11" t="s">
-        <v>354</v>
       </c>
       <c r="E82" s="8"/>
       <c r="F82" s="7"/>
       <c r="G82" s="11" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="409.6">
       <c r="A83" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="B83" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="B83" s="7" t="s">
+      <c r="C83" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="C83" s="7" t="s">
+      <c r="D83" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="D83" s="7" t="s">
+      <c r="E83" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="G83" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="E83" s="8" t="s">
+    </row>
+    <row r="84" spans="1:7" ht="409.6">
+      <c r="A84" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="E84" s="8" t="s">
         <v>485</v>
       </c>
-      <c r="F83" s="7" t="s">
-        <v>361</v>
-      </c>
-      <c r="G83" s="7" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" ht="314">
-      <c r="A84" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="B84" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="C84" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="D84" s="7" t="s">
+      <c r="F84" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="G84" s="7" t="s">
         <v>365</v>
-      </c>
-      <c r="E84" s="8" t="s">
-        <v>486</v>
-      </c>
-      <c r="F84" s="7" t="s">
-        <v>367</v>
-      </c>
-      <c r="G84" s="7" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="370">
       <c r="A85" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B85" s="7" t="s">
         <v>368</v>
       </c>
-      <c r="B85" s="7" t="s">
+      <c r="C85" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="C85" s="7" t="s">
+      <c r="D85" s="7" t="s">
         <v>370</v>
-      </c>
-      <c r="D85" s="7" t="s">
-        <v>371</v>
       </c>
       <c r="E85" s="8"/>
       <c r="F85" s="7"/>
       <c r="G85" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="195">
       <c r="A86" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="B86" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="B86" s="7" t="s">
+      <c r="C86" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="C86" s="7" t="s">
+      <c r="D86" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="D86" s="7" t="s">
-        <v>376</v>
-      </c>
       <c r="E86" s="8" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="F86" s="7"/>
       <c r="G86" s="7" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="105">
       <c r="A87" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="C87" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="B87" s="7" t="s">
-        <v>378</v>
-      </c>
-      <c r="C87" s="7" t="s">
+      <c r="D87" s="7" t="s">
         <v>379</v>
-      </c>
-      <c r="D87" s="7" t="s">
-        <v>380</v>
       </c>
       <c r="E87" s="8"/>
       <c r="F87" s="7"/>
@@ -4246,34 +4246,34 @@
     </row>
     <row r="88" spans="1:7" ht="105">
       <c r="A88" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="B88" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="B88" s="7" t="s">
+      <c r="C88" s="7" t="s">
         <v>382</v>
       </c>
-      <c r="C88" s="7" t="s">
+      <c r="D88" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="D88" s="7" t="s">
-        <v>384</v>
-      </c>
       <c r="E88" s="8" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F88" s="7"/>
       <c r="G88" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="409.6">
       <c r="A89" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B89" s="7" t="s">
         <v>386</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="C89" s="7" t="s">
         <v>387</v>
-      </c>
-      <c r="C89" s="7" t="s">
-        <v>388</v>
       </c>
       <c r="D89" s="7"/>
       <c r="E89" s="8"/>
@@ -4282,37 +4282,37 @@
     </row>
     <row r="90" spans="1:7" ht="409.6">
       <c r="A90" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="C90" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="B90" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="C90" s="7" t="s">
+      <c r="D90" s="7" t="s">
         <v>390</v>
       </c>
-      <c r="D90" s="7" t="s">
-        <v>391</v>
-      </c>
       <c r="E90" s="8" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F90" s="7"/>
       <c r="G90" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="126">
       <c r="A91" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C91" s="7" t="s">
         <v>393</v>
       </c>
-      <c r="B91" s="7" t="s">
-        <v>393</v>
-      </c>
-      <c r="C91" s="7" t="s">
+      <c r="D91" s="11" t="s">
         <v>394</v>
-      </c>
-      <c r="D91" s="11" t="s">
-        <v>395</v>
       </c>
       <c r="E91" s="8"/>
       <c r="F91" s="7"/>
@@ -4320,228 +4320,228 @@
     </row>
     <row r="92" spans="1:7" ht="150">
       <c r="A92" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="B92" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="C92" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="B92" s="7" t="s">
-        <v>396</v>
-      </c>
-      <c r="C92" s="7" t="s">
+      <c r="D92" s="7" t="s">
         <v>397</v>
-      </c>
-      <c r="D92" s="7" t="s">
-        <v>398</v>
       </c>
       <c r="E92" s="8"/>
       <c r="F92" s="7"/>
       <c r="G92" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="342">
       <c r="A93" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="C93" s="7" t="s">
         <v>400</v>
-      </c>
-      <c r="B93" s="7" t="s">
-        <v>400</v>
-      </c>
-      <c r="C93" s="7" t="s">
-        <v>401</v>
       </c>
       <c r="D93" s="7"/>
       <c r="E93" s="8" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F93" s="7"/>
       <c r="G93" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="285">
       <c r="A94" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="B94" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="C94" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="D94" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="D94" s="7" t="s">
-        <v>406</v>
-      </c>
       <c r="E94" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F94" s="7"/>
       <c r="G94" s="7" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="150">
       <c r="A95" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="C95" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="B95" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="C95" s="7" t="s">
+      <c r="D95" s="7" t="s">
         <v>409</v>
-      </c>
-      <c r="D95" s="7" t="s">
-        <v>410</v>
       </c>
       <c r="E95" s="8"/>
       <c r="F95" s="7"/>
       <c r="G95" s="7" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="135">
       <c r="A96" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="B96" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="B96" s="7" t="s">
+      <c r="C96" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="C96" s="7" t="s">
+      <c r="D96" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="D96" s="7" t="s">
-        <v>415</v>
-      </c>
       <c r="E96" s="8" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F96" s="7"/>
       <c r="G96" s="7" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="180">
       <c r="A97" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="B97" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="B97" s="7" t="s">
+      <c r="C97" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="C97" s="7" t="s">
+      <c r="D97" s="7" t="s">
         <v>419</v>
-      </c>
-      <c r="D97" s="7" t="s">
-        <v>420</v>
       </c>
       <c r="E97" s="8"/>
       <c r="F97" s="7"/>
       <c r="G97" s="7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="90">
       <c r="A98" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="B98" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="B98" s="7" t="s">
+      <c r="C98" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="C98" s="7" t="s">
+      <c r="D98" s="7" t="s">
         <v>424</v>
-      </c>
-      <c r="D98" s="7" t="s">
-        <v>425</v>
       </c>
       <c r="E98" s="8"/>
       <c r="F98" s="7"/>
       <c r="G98" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="409.6">
       <c r="A99" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="C99" s="7" t="s">
         <v>427</v>
       </c>
-      <c r="B99" s="7" t="s">
-        <v>427</v>
-      </c>
-      <c r="C99" s="7" t="s">
+      <c r="D99" s="7" t="s">
         <v>428</v>
       </c>
-      <c r="D99" s="7" t="s">
+      <c r="E99" s="8" t="s">
+        <v>492</v>
+      </c>
+      <c r="F99" s="7" t="s">
         <v>429</v>
-      </c>
-      <c r="E99" s="8" t="s">
-        <v>493</v>
-      </c>
-      <c r="F99" s="7" t="s">
-        <v>430</v>
       </c>
       <c r="G99" s="7"/>
     </row>
     <row r="100" spans="1:7" ht="409.6">
       <c r="A100" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="C100" s="7" t="s">
         <v>431</v>
       </c>
-      <c r="B100" s="7" t="s">
-        <v>431</v>
-      </c>
-      <c r="C100" s="7" t="s">
+      <c r="D100" s="7" t="s">
         <v>432</v>
       </c>
-      <c r="D100" s="7" t="s">
+      <c r="E100" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="F100" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="G100" s="7" t="s">
         <v>433</v>
-      </c>
-      <c r="E100" s="8" t="s">
-        <v>494</v>
-      </c>
-      <c r="F100" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="G100" s="7" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="356">
       <c r="A101" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="B101" s="7" t="s">
         <v>436</v>
       </c>
-      <c r="B101" s="7" t="s">
+      <c r="C101" s="7" t="s">
         <v>437</v>
-      </c>
-      <c r="C101" s="7" t="s">
-        <v>438</v>
       </c>
       <c r="D101" s="7"/>
       <c r="E101" s="8"/>
       <c r="F101" s="7"/>
       <c r="G101" s="7" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="135">
       <c r="A102" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="C102" s="7" t="s">
         <v>440</v>
-      </c>
-      <c r="B102" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="C102" s="7" t="s">
-        <v>441</v>
       </c>
       <c r="D102" s="7"/>
       <c r="E102" s="8"/>
       <c r="F102" s="7"/>
       <c r="G102" s="7" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="75">
       <c r="A103" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="C103" s="7" t="s">
         <v>443</v>
-      </c>
-      <c r="B103" s="7" t="s">
-        <v>443</v>
-      </c>
-      <c r="C103" s="7" t="s">
-        <v>444</v>
       </c>
       <c r="D103" s="7"/>
       <c r="E103" s="8"/>
@@ -4550,32 +4550,32 @@
     </row>
     <row r="104" spans="1:7" ht="105">
       <c r="A104" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="C104" s="7" t="s">
         <v>446</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="D104" s="7" t="s">
         <v>447</v>
-      </c>
-      <c r="D104" s="7" t="s">
-        <v>448</v>
       </c>
       <c r="E104" s="8"/>
       <c r="F104" s="7"/>
       <c r="G104" s="7" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="75">
       <c r="A105" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="B105" s="7" t="s">
         <v>450</v>
       </c>
-      <c r="B105" s="7" t="s">
+      <c r="C105" s="7" t="s">
         <v>451</v>
-      </c>
-      <c r="C105" s="7" t="s">
-        <v>452</v>
       </c>
       <c r="D105" s="7"/>
       <c r="E105" s="8"/>
@@ -4584,13 +4584,13 @@
     </row>
     <row r="106" spans="1:7" ht="75">
       <c r="A106" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="B106" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="B106" s="7" t="s">
+      <c r="C106" s="7" t="s">
         <v>454</v>
-      </c>
-      <c r="C106" s="7" t="s">
-        <v>455</v>
       </c>
       <c r="D106" s="7"/>
       <c r="E106" s="8"/>
@@ -4599,13 +4599,13 @@
     </row>
     <row r="107" spans="1:7" ht="105">
       <c r="A107" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="C107" s="7" t="s">
         <v>456</v>
-      </c>
-      <c r="B107" s="7" t="s">
-        <v>456</v>
-      </c>
-      <c r="C107" s="7" t="s">
-        <v>457</v>
       </c>
       <c r="D107" s="7"/>
       <c r="E107" s="8"/>
@@ -4614,34 +4614,34 @@
     </row>
     <row r="108" spans="1:7" ht="180">
       <c r="A108" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="B108" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="B108" s="7" t="s">
+      <c r="C108" s="7" t="s">
         <v>459</v>
       </c>
-      <c r="C108" s="7" t="s">
+      <c r="D108" s="7" t="s">
         <v>460</v>
       </c>
-      <c r="D108" s="7" t="s">
-        <v>461</v>
-      </c>
       <c r="E108" s="8" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F108" s="7"/>
       <c r="G108" s="7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="30">
       <c r="A109" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="C109" s="7" t="s">
         <v>463</v>
-      </c>
-      <c r="B109" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="C109" s="7" t="s">
-        <v>464</v>
       </c>
       <c r="D109" s="7"/>
       <c r="E109" s="8"/>
@@ -4650,59 +4650,59 @@
     </row>
     <row r="110" spans="1:7" ht="75">
       <c r="A110" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="C110" s="7" t="s">
         <v>465</v>
-      </c>
-      <c r="B110" s="7" t="s">
-        <v>465</v>
-      </c>
-      <c r="C110" s="7" t="s">
-        <v>466</v>
       </c>
       <c r="D110" s="7"/>
       <c r="E110" s="8" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F110" s="7"/>
       <c r="G110" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="105">
       <c r="A111" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="B111" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="B111" s="7" t="s">
+      <c r="C111" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="C111" s="7" t="s">
+      <c r="D111" s="7" t="s">
         <v>470</v>
-      </c>
-      <c r="D111" s="7" t="s">
-        <v>471</v>
       </c>
       <c r="E111" s="8"/>
       <c r="F111" s="7"/>
       <c r="G111" s="7" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="105">
       <c r="A112" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="B112" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="B112" s="7" t="s">
+      <c r="C112" s="7" t="s">
         <v>474</v>
       </c>
-      <c r="C112" s="7" t="s">
+      <c r="D112" s="7" t="s">
         <v>475</v>
-      </c>
-      <c r="D112" s="7" t="s">
-        <v>476</v>
       </c>
       <c r="E112" s="8"/>
       <c r="F112" s="7"/>
       <c r="G112" s="7" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="16">

</xml_diff>